<commit_message>
updated legacy GSC export data
</commit_message>
<xml_diff>
--- a/gsc-export-old/Coverage.xlsx
+++ b/gsc-export-old/Coverage.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="111">
   <si>
     <t>Date</t>
   </si>
@@ -29,18 +29,12 @@
     <t>Impressions</t>
   </si>
   <si>
-    <t>2025-11-23</t>
+    <t>2025-11-25</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>2025-11-24</t>
-  </si>
-  <si>
-    <t>2025-11-25</t>
-  </si>
-  <si>
     <t>2025-11-26</t>
   </si>
   <si>
@@ -291,6 +285,18 @@
   </si>
   <si>
     <t>2026-02-17</t>
+  </si>
+  <si>
+    <t>2026-02-18</t>
+  </si>
+  <si>
+    <t>2026-02-19</t>
+  </si>
+  <si>
+    <t>2026-02-20</t>
+  </si>
+  <si>
+    <t>2026-02-21</t>
   </si>
   <si>
     <t>Reason</t>
@@ -391,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -419,7 +425,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>9.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="3">
@@ -433,7 +439,7 @@
         <v>5</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="4">
@@ -447,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>14.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="5">
@@ -461,7 +467,7 @@
         <v>5</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="6">
@@ -475,7 +481,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
@@ -489,7 +495,7 @@
         <v>5</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>2.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +509,7 @@
         <v>5</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +523,7 @@
         <v>5</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>7.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="10">
@@ -531,7 +537,7 @@
         <v>5</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11">
@@ -545,7 +551,7 @@
         <v>5</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>4.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="12">
@@ -559,7 +565,7 @@
         <v>5</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
@@ -573,7 +579,7 @@
         <v>5</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="14">
@@ -587,7 +593,7 @@
         <v>5</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="15">
@@ -601,7 +607,7 @@
         <v>5</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="16">
@@ -615,7 +621,7 @@
         <v>5</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="17">
@@ -629,7 +635,7 @@
         <v>5</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="18">
@@ -657,7 +663,7 @@
         <v>5</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="20">
@@ -671,7 +677,7 @@
         <v>5</v>
       </c>
       <c r="D20" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="21">
@@ -685,35 +691,35 @@
         <v>5</v>
       </c>
       <c r="D21" t="n" s="0">
-        <v>3.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="B22" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="C22" t="s" s="0">
-        <v>5</v>
+      <c r="B22" t="n" s="0">
+        <v>73.0</v>
+      </c>
+      <c r="C22" t="n" s="0">
+        <v>62.0</v>
       </c>
       <c r="D22" t="n" s="0">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="B23" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="C23" t="s" s="0">
-        <v>5</v>
+      <c r="B23" t="n" s="0">
+        <v>79.0</v>
+      </c>
+      <c r="C23" t="n" s="0">
+        <v>56.0</v>
       </c>
       <c r="D23" t="n" s="0">
-        <v>16.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="24">
@@ -721,13 +727,13 @@
         <v>27</v>
       </c>
       <c r="B24" t="n" s="0">
-        <v>73.0</v>
+        <v>79.0</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>62.0</v>
+        <v>56.0</v>
       </c>
       <c r="D24" t="n" s="0">
-        <v>4.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="25">
@@ -741,7 +747,7 @@
         <v>56.0</v>
       </c>
       <c r="D25" t="n" s="0">
-        <v>9.0</v>
+        <v>15.0</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +761,7 @@
         <v>56.0</v>
       </c>
       <c r="D26" t="n" s="0">
-        <v>9.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="27">
@@ -769,7 +775,7 @@
         <v>56.0</v>
       </c>
       <c r="D27" t="n" s="0">
-        <v>15.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="28">
@@ -783,7 +789,7 @@
         <v>56.0</v>
       </c>
       <c r="D28" t="n" s="0">
-        <v>7.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="29">
@@ -797,7 +803,7 @@
         <v>56.0</v>
       </c>
       <c r="D29" t="n" s="0">
-        <v>7.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="30">
@@ -811,7 +817,7 @@
         <v>56.0</v>
       </c>
       <c r="D30" t="n" s="0">
-        <v>3.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="31">
@@ -819,13 +825,13 @@
         <v>34</v>
       </c>
       <c r="B31" t="n" s="0">
-        <v>79.0</v>
+        <v>85.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>56.0</v>
+        <v>50.0</v>
       </c>
       <c r="D31" t="n" s="0">
-        <v>12.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="32">
@@ -833,13 +839,13 @@
         <v>35</v>
       </c>
       <c r="B32" t="n" s="0">
-        <v>79.0</v>
+        <v>85.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>56.0</v>
+        <v>50.0</v>
       </c>
       <c r="D32" t="n" s="0">
-        <v>2.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="33">
@@ -853,7 +859,7 @@
         <v>50.0</v>
       </c>
       <c r="D33" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="34">
@@ -867,7 +873,7 @@
         <v>50.0</v>
       </c>
       <c r="D34" t="n" s="0">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="35">
@@ -895,7 +901,7 @@
         <v>50.0</v>
       </c>
       <c r="D36" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="37">
@@ -909,7 +915,7 @@
         <v>50.0</v>
       </c>
       <c r="D37" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="38">
@@ -923,7 +929,7 @@
         <v>50.0</v>
       </c>
       <c r="D38" t="n" s="0">
-        <v>0.0</v>
+        <v>72.0</v>
       </c>
     </row>
     <row r="39">
@@ -951,7 +957,7 @@
         <v>50.0</v>
       </c>
       <c r="D40" t="n" s="0">
-        <v>72.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="41">
@@ -965,7 +971,7 @@
         <v>50.0</v>
       </c>
       <c r="D41" t="n" s="0">
-        <v>1.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="42">
@@ -973,13 +979,13 @@
         <v>45</v>
       </c>
       <c r="B42" t="n" s="0">
-        <v>85.0</v>
+        <v>90.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="D42" t="n" s="0">
-        <v>2.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="43">
@@ -987,13 +993,13 @@
         <v>46</v>
       </c>
       <c r="B43" t="n" s="0">
-        <v>85.0</v>
+        <v>90.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="D43" t="n" s="0">
-        <v>29.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="44">
@@ -1007,7 +1013,7 @@
         <v>45.0</v>
       </c>
       <c r="D44" t="n" s="0">
-        <v>10.0</v>
+        <v>29.0</v>
       </c>
     </row>
     <row r="45">
@@ -1015,13 +1021,13 @@
         <v>48</v>
       </c>
       <c r="B45" t="n" s="0">
-        <v>90.0</v>
+        <v>93.0</v>
       </c>
       <c r="C45" t="n" s="0">
-        <v>45.0</v>
+        <v>42.0</v>
       </c>
       <c r="D45" t="n" s="0">
-        <v>2.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="46">
@@ -1029,13 +1035,13 @@
         <v>49</v>
       </c>
       <c r="B46" t="n" s="0">
-        <v>90.0</v>
+        <v>93.0</v>
       </c>
       <c r="C46" t="n" s="0">
-        <v>45.0</v>
+        <v>42.0</v>
       </c>
       <c r="D46" t="n" s="0">
-        <v>29.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="47">
@@ -1049,7 +1055,7 @@
         <v>42.0</v>
       </c>
       <c r="D47" t="n" s="0">
-        <v>40.0</v>
+        <v>85.0</v>
       </c>
     </row>
     <row r="48">
@@ -1063,7 +1069,7 @@
         <v>42.0</v>
       </c>
       <c r="D48" t="n" s="0">
-        <v>14.0</v>
+        <v>121.0</v>
       </c>
     </row>
     <row r="49">
@@ -1071,13 +1077,13 @@
         <v>52</v>
       </c>
       <c r="B49" t="n" s="0">
-        <v>93.0</v>
+        <v>94.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>42.0</v>
+        <v>41.0</v>
       </c>
       <c r="D49" t="n" s="0">
-        <v>85.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="50">
@@ -1085,13 +1091,13 @@
         <v>53</v>
       </c>
       <c r="B50" t="n" s="0">
-        <v>93.0</v>
+        <v>94.0</v>
       </c>
       <c r="C50" t="n" s="0">
-        <v>42.0</v>
+        <v>41.0</v>
       </c>
       <c r="D50" t="n" s="0">
-        <v>121.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="51">
@@ -1105,7 +1111,7 @@
         <v>41.0</v>
       </c>
       <c r="D51" t="n" s="0">
-        <v>9.0</v>
+        <v>67.0</v>
       </c>
     </row>
     <row r="52">
@@ -1113,13 +1119,13 @@
         <v>55</v>
       </c>
       <c r="B52" t="n" s="0">
-        <v>94.0</v>
+        <v>95.0</v>
       </c>
       <c r="C52" t="n" s="0">
-        <v>41.0</v>
+        <v>40.0</v>
       </c>
       <c r="D52" t="n" s="0">
-        <v>26.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="53">
@@ -1127,13 +1133,13 @@
         <v>56</v>
       </c>
       <c r="B53" t="n" s="0">
-        <v>94.0</v>
+        <v>95.0</v>
       </c>
       <c r="C53" t="n" s="0">
-        <v>41.0</v>
+        <v>40.0</v>
       </c>
       <c r="D53" t="n" s="0">
-        <v>67.0</v>
+        <v>25.0</v>
       </c>
     </row>
     <row r="54">
@@ -1147,7 +1153,7 @@
         <v>40.0</v>
       </c>
       <c r="D54" t="n" s="0">
-        <v>54.0</v>
+        <v>23.0</v>
       </c>
     </row>
     <row r="55">
@@ -1161,7 +1167,7 @@
         <v>40.0</v>
       </c>
       <c r="D55" t="n" s="0">
-        <v>25.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="56">
@@ -1169,13 +1175,13 @@
         <v>59</v>
       </c>
       <c r="B56" t="n" s="0">
-        <v>95.0</v>
+        <v>101.0</v>
       </c>
       <c r="C56" t="n" s="0">
-        <v>40.0</v>
+        <v>34.0</v>
       </c>
       <c r="D56" t="n" s="0">
-        <v>23.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="57">
@@ -1183,13 +1189,13 @@
         <v>60</v>
       </c>
       <c r="B57" t="n" s="0">
-        <v>95.0</v>
+        <v>101.0</v>
       </c>
       <c r="C57" t="n" s="0">
-        <v>40.0</v>
+        <v>34.0</v>
       </c>
       <c r="D57" t="n" s="0">
-        <v>33.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="58">
@@ -1203,7 +1209,7 @@
         <v>34.0</v>
       </c>
       <c r="D58" t="n" s="0">
-        <v>3.0</v>
+        <v>44.0</v>
       </c>
     </row>
     <row r="59">
@@ -1217,7 +1223,7 @@
         <v>34.0</v>
       </c>
       <c r="D59" t="n" s="0">
-        <v>13.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="60">
@@ -1231,7 +1237,7 @@
         <v>34.0</v>
       </c>
       <c r="D60" t="n" s="0">
-        <v>44.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="61">
@@ -1245,7 +1251,7 @@
         <v>34.0</v>
       </c>
       <c r="D61" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="62">
@@ -1259,7 +1265,7 @@
         <v>34.0</v>
       </c>
       <c r="D62" t="n" s="0">
-        <v>0.0</v>
+        <v>58.0</v>
       </c>
     </row>
     <row r="63">
@@ -1267,13 +1273,13 @@
         <v>66</v>
       </c>
       <c r="B63" t="n" s="0">
-        <v>101.0</v>
+        <v>104.0</v>
       </c>
       <c r="C63" t="n" s="0">
-        <v>34.0</v>
+        <v>31.0</v>
       </c>
       <c r="D63" t="n" s="0">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="64">
@@ -1281,13 +1287,13 @@
         <v>67</v>
       </c>
       <c r="B64" t="n" s="0">
-        <v>101.0</v>
+        <v>104.0</v>
       </c>
       <c r="C64" t="n" s="0">
-        <v>34.0</v>
+        <v>31.0</v>
       </c>
       <c r="D64" t="n" s="0">
-        <v>58.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="65">
@@ -1301,7 +1307,7 @@
         <v>31.0</v>
       </c>
       <c r="D65" t="n" s="0">
-        <v>4.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="66">
@@ -1309,13 +1315,13 @@
         <v>69</v>
       </c>
       <c r="B66" t="n" s="0">
-        <v>104.0</v>
+        <v>106.0</v>
       </c>
       <c r="C66" t="n" s="0">
-        <v>31.0</v>
+        <v>29.0</v>
       </c>
       <c r="D66" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="67">
@@ -1323,13 +1329,13 @@
         <v>70</v>
       </c>
       <c r="B67" t="n" s="0">
-        <v>104.0</v>
+        <v>106.0</v>
       </c>
       <c r="C67" t="n" s="0">
-        <v>31.0</v>
+        <v>29.0</v>
       </c>
       <c r="D67" t="n" s="0">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="68">
@@ -1343,7 +1349,7 @@
         <v>29.0</v>
       </c>
       <c r="D68" t="n" s="0">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="69">
@@ -1357,7 +1363,7 @@
         <v>29.0</v>
       </c>
       <c r="D69" t="n" s="0">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="70">
@@ -1365,13 +1371,13 @@
         <v>73</v>
       </c>
       <c r="B70" t="n" s="0">
-        <v>106.0</v>
+        <v>110.0</v>
       </c>
       <c r="C70" t="n" s="0">
-        <v>29.0</v>
+        <v>25.0</v>
       </c>
       <c r="D70" t="n" s="0">
-        <v>6.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="71">
@@ -1379,10 +1385,10 @@
         <v>74</v>
       </c>
       <c r="B71" t="n" s="0">
-        <v>106.0</v>
+        <v>110.0</v>
       </c>
       <c r="C71" t="n" s="0">
-        <v>29.0</v>
+        <v>25.0</v>
       </c>
       <c r="D71" t="n" s="0">
         <v>0.0</v>
@@ -1407,13 +1413,13 @@
         <v>76</v>
       </c>
       <c r="B73" t="n" s="0">
-        <v>110.0</v>
+        <v>114.0</v>
       </c>
       <c r="C73" t="n" s="0">
-        <v>25.0</v>
+        <v>21.0</v>
       </c>
       <c r="D73" t="n" s="0">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="74">
@@ -1421,13 +1427,13 @@
         <v>77</v>
       </c>
       <c r="B74" t="n" s="0">
-        <v>110.0</v>
+        <v>114.0</v>
       </c>
       <c r="C74" t="n" s="0">
-        <v>25.0</v>
+        <v>21.0</v>
       </c>
       <c r="D74" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="75">
@@ -1441,7 +1447,7 @@
         <v>21.0</v>
       </c>
       <c r="D75" t="n" s="0">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
     </row>
     <row r="76">
@@ -1455,7 +1461,7 @@
         <v>21.0</v>
       </c>
       <c r="D76" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="77">
@@ -1463,13 +1469,13 @@
         <v>80</v>
       </c>
       <c r="B77" t="n" s="0">
-        <v>114.0</v>
+        <v>121.0</v>
       </c>
       <c r="C77" t="n" s="0">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
       <c r="D77" t="n" s="0">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="78">
@@ -1477,10 +1483,10 @@
         <v>81</v>
       </c>
       <c r="B78" t="n" s="0">
-        <v>114.0</v>
+        <v>121.0</v>
       </c>
       <c r="C78" t="n" s="0">
-        <v>21.0</v>
+        <v>14.0</v>
       </c>
       <c r="D78" t="n" s="0">
         <v>0.0</v>
@@ -1497,7 +1503,7 @@
         <v>14.0</v>
       </c>
       <c r="D79" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="80">
@@ -1505,13 +1511,13 @@
         <v>83</v>
       </c>
       <c r="B80" t="n" s="0">
-        <v>121.0</v>
+        <v>135.0</v>
       </c>
       <c r="C80" t="n" s="0">
-        <v>14.0</v>
+        <v>0.0</v>
       </c>
       <c r="D80" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="81">
@@ -1519,10 +1525,10 @@
         <v>84</v>
       </c>
       <c r="B81" t="n" s="0">
-        <v>121.0</v>
+        <v>135.0</v>
       </c>
       <c r="C81" t="n" s="0">
-        <v>14.0</v>
+        <v>0.0</v>
       </c>
       <c r="D81" t="n" s="0">
         <v>0.0</v>
@@ -1539,7 +1545,7 @@
         <v>0.0</v>
       </c>
       <c r="D82" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="83">
@@ -1624,6 +1630,34 @@
       </c>
       <c r="D88" t="n" s="0">
         <v>0.0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="B89" t="n" s="0">
+        <v>135.0</v>
+      </c>
+      <c r="C89" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D89" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="B90" t="n" s="0">
+        <v>135.0</v>
+      </c>
+      <c r="C90" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1638,41 +1672,41 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>103.0</v>
+        <v>104.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
+        <v>101</v>
+      </c>
+      <c r="B3" t="s" s="0">
         <v>99</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>97</v>
-      </c>
       <c r="C3" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n" s="0">
         <v>4.0</v>
@@ -1680,13 +1714,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>102</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>100</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>97</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>98</v>
       </c>
       <c r="D4" t="n" s="0">
         <v>3.0</v>
@@ -1694,13 +1728,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D5" t="n" s="0">
         <v>15.0</v>
@@ -1708,16 +1742,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>10.0</v>
+        <v>9.0</v>
       </c>
     </row>
   </sheetData>
@@ -1732,16 +1766,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1756,18 +1790,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>